<commit_message>
vulns_framework_mapping.xlsx: show lockout-threshold override on vuln 27
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vulns_framework_mapping.xlsx
+++ b/vulns_framework_mapping.xlsx
@@ -1428,13 +1428,34 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>No Account Lockout Policy (threshold &gt; 5)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>CIS 5.2
+CIS 6.5</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1.4.1</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>8.3.4</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>IAC-06</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -3815,7 +3836,8 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Account Lockout Duration Not Configured Or Insufficient</t>
+          <t>Account Lockout Duration Not Configured Or Insufficient
+(threshold &gt; 5 → 27: Excessive Number Of Failed Login Attempts Allowed)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">

</xml_diff>

<commit_message>
vulns.txt: add 'User-ID Is Not Turned On / Configured' (60) and 'Server Verification Disabled' (61); map PA User-ID / update-server findings to them
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vulns_framework_mapping.xlsx
+++ b/vulns_framework_mapping.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Finding" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By Vuln'!$A$1:$H$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By Vuln'!$A$1:$H$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'By Finding'!$A$1:$G$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2499,8 +2499,81 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>User-ID Is Not Turned On / Configured</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>User-ID Not Configured</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>CIS 6.1</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>IAC-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Server Verification Disabled</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Update Server Verification Disabled</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>CIS 4.6
+CIS 12.6</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>6.3.1</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>VPM-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H60"/>
+  <autoFilter ref="A1:H62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4942,10 +5015,12 @@
           <t>Update Server Verification Disabled</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr"/>
+      <c r="B75" s="2" t="n">
+        <v>61</v>
+      </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>(not mapped)</t>
+          <t>Server Verification Disabled</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -5107,10 +5182,12 @@
           <t>User-ID Not Configured</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr"/>
+      <c r="B80" s="2" t="n">
+        <v>60</v>
+      </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>(not mapped)</t>
+          <t>User-ID Is Not Turned On / Configured</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">

</xml_diff>

<commit_message>
SCF mappings: move PA and Check Point analyzers to SCF 2026.3 IDs at sub-control level (e.g. IAC-15.1, CFG-04.1, NET-04.1); regenerate mapping workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vulns_framework_mapping.xlsx
+++ b/vulns_framework_mapping.xlsx
@@ -555,7 +555,8 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11.1
+SEA-30</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
@@ -603,7 +604,9 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14
+IAC-14.4
+IAC-15</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
@@ -679,7 +682,7 @@
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>AST-03</t>
         </is>
       </c>
     </row>
@@ -703,7 +706,12 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>CFG-08
+NET-04.2</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="n">
         <v>2</v>
       </c>
@@ -726,7 +734,7 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>NET-04.2</t>
         </is>
       </c>
     </row>
@@ -787,8 +795,8 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-OPS-01</t>
+          <t>CRY-06
+MON-11.1</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
@@ -838,8 +846,8 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>TDA-02
-VPM-10</t>
+          <t>THR-04
+VPM-08.1</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
@@ -891,8 +899,9 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-IAC-10</t>
+          <t>CFG-04.7
+CRY-09
+CRY-12</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -939,7 +948,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
@@ -967,7 +976,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1041,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
@@ -1056,7 +1065,7 @@
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1103,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
@@ -1123,8 +1132,8 @@
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>IAC-06
-IAC-07</t>
+          <t>IAC-08.4
+IAC-14.1</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1197,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
@@ -1212,7 +1221,7 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1285,8 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-03
+CRY-05</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
@@ -1311,7 +1321,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1359,8 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>NET-20.1
+NET-42.2</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
@@ -1401,9 +1412,10 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>NET-04
-NET-14
-TDA-02</t>
+          <t>NET-03.9
+NET-17
+NET-31
+THR-04</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
@@ -1458,8 +1470,8 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>IAC-06
-NET-04</t>
+          <t>IAC-14.2
+NET-17</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
@@ -1506,7 +1518,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>DAM-01</t>
+          <t>NET-03.5</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
@@ -1587,11 +1599,16 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-NET-04
-NET-14
-TDA-02
-VPM-01</t>
+          <t>END-04
+END-04.1
+END-04.2
+MON-09
+NET-03.6
+NET-20
+NET-20.1
+NET-21
+NET-31
+NET-42.2</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
@@ -1637,7 +1654,8 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>CFG-04.3
+CFG-04.5</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
@@ -1663,7 +1681,7 @@
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>CFG-04.5</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1716,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-05</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
@@ -1723,7 +1741,7 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-05</t>
         </is>
       </c>
     </row>
@@ -1770,8 +1788,9 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>IAC-10
-NET-04</t>
+          <t>NET-03
+NET-04.1
+NET-26.1</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
@@ -1800,7 +1819,7 @@
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1861,8 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03
+NET-04.1</t>
         </is>
       </c>
       <c r="I27" s="2" t="n">
@@ -1868,7 +1888,7 @@
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1927,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
@@ -1937,7 +1957,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
     </row>
@@ -1982,7 +2002,9 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1
+IAC-15
+IAC-15.1</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
@@ -2008,7 +2030,7 @@
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2072,7 @@
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1</t>
         </is>
       </c>
     </row>
@@ -2129,9 +2151,10 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>NET-14
-TDA-02
-VPM-01</t>
+          <t>END-04
+NET-03
+NET-31
+NET-42.2</t>
         </is>
       </c>
       <c r="I32" s="2" t="n">
@@ -2194,8 +2217,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>MON-06
-TDA-02</t>
+          <t>MON-04
+MON-05
+MON-05.5
+MON-09
+MON-22.1
+MON-31</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
@@ -2239,8 +2266,11 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>MON-06
-NET-04</t>
+          <t>MON-04
+MON-13
+MON-14
+MON-31
+NET-04.2</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2312,9 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04
+CRY-05
+CRY-06</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
@@ -2325,7 +2357,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="I35" s="2" t="n">
@@ -2367,7 +2399,8 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04
+CRY-05</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
@@ -2409,7 +2442,8 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-08
+NET-04.2</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
@@ -2429,7 +2463,8 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-08
+NET-04.2</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2498,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
@@ -2488,7 +2523,7 @@
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-04.2</t>
         </is>
       </c>
     </row>
@@ -2522,8 +2557,8 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-MON-06</t>
+          <t>CRY-05
+MON-12.3</t>
         </is>
       </c>
       <c r="I39" s="2" t="n">
@@ -2576,10 +2611,13 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>CRY-01
-IAC-01
-IAC-07
-IAC-10</t>
+          <t>CRY-10
+IAC-03
+IAC-10
+IAC-25
+IAC-30
+IAC-32
+IAC-34</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
@@ -2609,8 +2647,9 @@
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>IAC-01
-IAC-07</t>
+          <t>IAC-03
+IAC-08.4
+IAC-32</t>
         </is>
       </c>
     </row>
@@ -2652,8 +2691,8 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-NET-06</t>
+          <t>CFG-04.7
+CRY-05</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -2684,7 +2723,8 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-04.7
+CRY-05</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2823,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
     </row>
@@ -2825,8 +2865,8 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>IAC-01
-NET-04</t>
+          <t>NET-04.1
+NET-09</t>
         </is>
       </c>
       <c r="I45" s="2" t="n">
@@ -2860,7 +2900,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2968,7 @@
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>SEA-28</t>
         </is>
       </c>
     </row>
@@ -2967,8 +3007,8 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-MON-06</t>
+          <t>CFG-04.7
+CRY-05</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
@@ -3014,7 +3054,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>SEA-28</t>
         </is>
       </c>
       <c r="I49" s="2" t="n">
@@ -3038,7 +3078,7 @@
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>SEA-28</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3112,7 @@
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>OPS-04</t>
+          <t>BCD-22</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
@@ -3174,8 +3214,9 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>IAC-10
-NET-04</t>
+          <t>NET-04.1
+NET-06.1
+NET-09</t>
         </is>
       </c>
       <c r="I53" s="2" t="n">
@@ -3212,8 +3253,8 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>IAC-10
-NET-04</t>
+          <t>NET-06.1
+NET-09</t>
         </is>
       </c>
     </row>
@@ -3250,8 +3291,8 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-NET-06</t>
+          <t>CFG-04.7
+CRY-05</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
@@ -3283,8 +3324,9 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>CRY-03
-NET-06</t>
+          <t>CFG-03
+CFG-04.7
+CRY-05</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3382,7 @@
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-13</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
@@ -3364,7 +3406,7 @@
       <c r="M56" s="2" t="inlineStr"/>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-13</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3440,8 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11.1
+SEA-30</t>
         </is>
       </c>
       <c r="I57" s="2" t="n">
@@ -3429,7 +3472,8 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11.1
+SEA-30</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3515,7 @@
       <c r="M58" s="2" t="inlineStr"/>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11</t>
         </is>
       </c>
     </row>
@@ -3517,8 +3561,8 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>IAC-01
-NET-04</t>
+          <t>CFG-03
+IAC-14.2</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
@@ -3562,7 +3606,8 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>IAC-30
+NET-04.1</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
@@ -3604,7 +3649,8 @@
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>IAC-01</t>
+          <t>IAC-25
+NET-14</t>
         </is>
       </c>
       <c r="I61" s="2" t="n">
@@ -3651,7 +3697,8 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>VPM-10</t>
+          <t>CHG-13
+VPM-08.2</t>
         </is>
       </c>
       <c r="I62" s="2" t="n">
@@ -3761,7 +3808,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>TDA-02 · VPM-10</t>
+          <t>THR-04 · VPM-08.1</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -3793,7 +3840,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14 · IAC-15</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -3829,7 +3876,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · IAC-10</t>
+          <t>CFG-04.7 · CRY-12</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -3861,7 +3908,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>IAC-01</t>
+          <t>IAC-03 · IAC-32</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -3897,7 +3944,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>NET-14 · TDA-02</t>
+          <t>END-04.2 · NET-31</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -3929,7 +3976,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-09 · MON-31</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -3965,7 +4012,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>NET-31</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -4001,7 +4048,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>NET-14 · TDA-02</t>
+          <t>NET-17 · NET-31</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -4037,7 +4084,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>END-04</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -4073,7 +4120,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>TDA-02 · VPM-01</t>
+          <t>END-04 · END-04.1</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -4105,7 +4152,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>IAC-30 · NET-04.1</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -4137,7 +4184,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03 · NET-04.1</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -4169,7 +4216,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-03 · CRY-05</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -4197,7 +4244,7 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-13</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -4233,7 +4280,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>DAM-01</t>
+          <t>NET-03.5</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -4269,7 +4316,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-09 · CRY-12</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -4305,7 +4352,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-31</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4337,7 +4384,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.4</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4369,7 +4416,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-08 · NET-04.2</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4401,7 +4448,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>IAC-07</t>
+          <t>IAC-10 · IAC-30</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4433,7 +4480,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>IAC-10 · NET-04</t>
+          <t>NET-04.1 · NET-26.1</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -4465,7 +4512,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>END-04</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -4501,7 +4548,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · NET-06</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -4533,7 +4580,7 @@
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>OPS-04</t>
+          <t>BCD-22</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -4569,7 +4616,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-04</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -4601,7 +4648,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>CRY-01</t>
+          <t>CRY-10 · IAC-34</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -4633,7 +4680,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -4665,7 +4712,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-05</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -4697,7 +4744,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>NET-14</t>
+          <t>NET-03 · NET-31</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -4729,7 +4776,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-03 · CRY-05</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -4765,7 +4812,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -4801,7 +4848,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>CFG-04.3 · CFG-04.5</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -4837,7 +4884,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>IAC-10 · NET-04</t>
+          <t>NET-06.1 · NET-09</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -4869,7 +4916,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -4901,7 +4948,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>NET-14</t>
+          <t>END-04 · NET-31</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -4933,7 +4980,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · OPS-01</t>
+          <t>CRY-06 · MON-11.1</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -4965,7 +5012,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11.1 · SEA-30</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -4997,7 +5044,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -5029,7 +5076,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -5065,7 +5112,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -5101,7 +5148,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -5137,7 +5184,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -5169,7 +5216,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-04 · MON-31</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -5205,7 +5252,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>SEA-28</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -5237,7 +5284,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>IAC-10 · NET-04</t>
+          <t>NET-06.1 · NET-09</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -5269,7 +5316,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-05</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -5301,7 +5348,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11.1 · SEA-30</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -5337,7 +5384,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03.6 · NET-21</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -5373,7 +5420,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15 · IAC-15.1</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -5409,7 +5456,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -5445,7 +5492,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1 · IAC-15</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -5477,7 +5524,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -5513,7 +5560,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-31</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -5545,7 +5592,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>IAC-01 · IAC-10</t>
+          <t>IAC-25 · IAC-30</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -5577,7 +5624,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03 · NET-04.1</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -5609,7 +5656,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1 · NET-09</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -5641,7 +5688,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · NET-06</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -5673,7 +5720,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · NET-06</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -5709,7 +5756,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · MON-06</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -5745,7 +5792,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-04 · MON-05</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -5777,7 +5824,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1 · NET-26.1</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -5813,7 +5860,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · NET-14</t>
+          <t>NET-20 · NET-20.1</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -5849,7 +5896,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03 · NET-04.1</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -5881,7 +5928,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · MON-06</t>
+          <t>CRY-05 · MON-12.3</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -5913,7 +5960,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-09 · CRY-12</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -5949,7 +5996,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · NET-06</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -5985,7 +6032,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>NET-04 · TDA-02</t>
+          <t>NET-03.9 · THR-04</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -6021,7 +6068,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-17</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -6057,7 +6104,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-17</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -6093,7 +6140,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-22.1</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -6129,7 +6176,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-17</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -6161,7 +6208,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -6193,7 +6240,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -6215,7 +6262,11 @@
       <c r="D75" s="2" t="inlineStr"/>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>CFG-08 · NET-04.2</t>
+        </is>
+      </c>
       <c r="H75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
@@ -6249,7 +6300,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>VPM-10</t>
+          <t>CHG-13 · VPM-08.2</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -6285,7 +6336,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>IAC-06 · NET-04</t>
+          <t>IAC-14.2 · NET-17</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -6321,7 +6372,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>IAC-01 · NET-04</t>
+          <t>NET-04.1 · NET-09</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -6353,7 +6404,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>IAC-01 · NET-04</t>
+          <t>CFG-03 · IAC-14.2</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -6385,7 +6436,7 @@
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>IAC-01 · NET-04</t>
+          <t>CFG-03 · IAC-14.2</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -6417,7 +6468,7 @@
       <c r="F81" s="2" t="inlineStr"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>IAC-01</t>
+          <t>IAC-25 · NET-14</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -6449,7 +6500,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1 · NET-26.1</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -6485,7 +6536,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>VPM-01</t>
+          <t>NET-31</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -6521,7 +6572,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>VPM-01</t>
+          <t>NET-31</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -6557,7 +6608,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>IAC-01 · NET-04</t>
+          <t>CFG-03 · IAC-14.2</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -6589,7 +6640,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-05</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -6621,7 +6672,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-05</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -6653,7 +6704,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-06</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr"/>
@@ -6685,7 +6736,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-06</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr"/>
@@ -6717,7 +6768,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-05</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr"/>
@@ -6749,7 +6800,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-05</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr"/>
@@ -6781,7 +6832,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CRY-04 · CRY-05</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr"/>
@@ -6817,7 +6868,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr"/>
@@ -6853,7 +6904,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>NET-20.1 · NET-42.2</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
@@ -6889,7 +6940,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>END-04.2 · NET-42.2</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr"/>
@@ -6925,7 +6976,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>END-04.2</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr"/>
@@ -6961,7 +7012,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>MON-05.5</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr"/>
@@ -6993,7 +7044,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>END-04.2 · NET-42.2</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr"/>
@@ -7025,7 +7076,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>END-04.2 · NET-42.2</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
@@ -7061,7 +7112,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>NET-42.2</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
@@ -7097,7 +7148,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>TDA-02</t>
+          <t>MON-09 · NET-42.2</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr"/>
@@ -7133,7 +7184,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>TDA-02 · VPM-10</t>
+          <t>THR-04 · VPM-08.1</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr"/>
@@ -7169,7 +7220,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-21</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
@@ -7201,7 +7252,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03.6 · NET-21</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr"/>
@@ -7300,7 +7351,7 @@
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -7336,7 +7387,7 @@
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -7372,7 +7423,7 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15.1</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -7408,7 +7459,7 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-15</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -7444,7 +7495,7 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -7480,7 +7531,7 @@
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -7516,7 +7567,7 @@
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>IAC-07</t>
+          <t>IAC-08.4</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -7552,7 +7603,7 @@
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>IAC-07</t>
+          <t>IAC-08.4</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -7588,7 +7639,7 @@
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>IAC-07</t>
+          <t>IAC-08.4</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -7624,7 +7675,7 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>IAC-14.1</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -7664,7 +7715,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -7704,7 +7755,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -7744,7 +7795,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>IAC-06</t>
+          <t>CFG-04.1</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -7780,7 +7831,7 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>SEA-28</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -7816,7 +7867,7 @@
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>SEA-28</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -7850,7 +7901,7 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>CFG-04</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -7884,7 +7935,7 @@
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>CFG-09</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -7924,7 +7975,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -7960,7 +8011,7 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-13</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -7998,7 +8049,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -8034,7 +8085,7 @@
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>AST-03</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -8074,7 +8125,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -8112,7 +8163,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -8152,7 +8203,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>CRY-03 · NET-06</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -8188,7 +8239,7 @@
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -8224,7 +8275,7 @@
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-04</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -8260,7 +8311,7 @@
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-05</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -8300,7 +8351,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11.1 · SEA-30</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -8336,7 +8387,7 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>MON-11</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -8370,7 +8421,7 @@
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>BCD-01</t>
+          <t>BCD-24</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -8404,7 +8455,7 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>BCD-01</t>
+          <t>BCD-24 · CFG-09</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -8438,7 +8489,7 @@
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>BCD-01</t>
+          <t>BCD-24</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -8474,7 +8525,7 @@
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>CFG-04.5</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -8510,7 +8561,7 @@
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>IAC-09</t>
+          <t>CFG-04.5</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -8546,7 +8597,7 @@
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>CRY-03</t>
+          <t>CFG-04.7 · CRY-05</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -8582,7 +8633,7 @@
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>IAC-01</t>
+          <t>IAC-03 · IAC-32</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -8622,7 +8673,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>IAC-10 · NET-04</t>
+          <t>NET-06.1 · NET-09</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -8658,7 +8709,7 @@
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-14</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -8694,7 +8745,7 @@
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-13</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -8730,7 +8781,7 @@
       <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-04</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -8770,7 +8821,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-09</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -8810,7 +8861,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -8846,7 +8897,7 @@
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -8882,7 +8933,7 @@
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -8918,7 +8969,7 @@
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -8954,7 +9005,7 @@
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -8990,7 +9041,7 @@
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -9030,7 +9081,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-31</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -9066,7 +9117,7 @@
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>MON-31 · NET-04.2</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -9100,7 +9151,7 @@
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03.6</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -9134,7 +9185,7 @@
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03.6</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -9168,7 +9219,7 @@
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -9202,7 +9253,7 @@
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-10.1</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -9238,7 +9289,7 @@
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -9274,7 +9325,7 @@
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -9310,7 +9361,7 @@
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -9350,7 +9401,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-03</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -9384,7 +9435,7 @@
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03.3</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -9418,7 +9469,7 @@
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-03.3</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -9454,7 +9505,7 @@
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-31</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -9486,7 +9537,7 @@
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>CFG-08 · NET-04.2</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -9518,7 +9569,7 @@
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -9554,7 +9605,7 @@
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -9590,7 +9641,7 @@
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -9626,7 +9677,7 @@
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -9666,7 +9717,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>MON-31</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -9702,7 +9753,7 @@
       <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>MON-06</t>
+          <t>NET-04.2</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -9742,7 +9793,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>NET-04</t>
+          <t>NET-04.1</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">

</xml_diff>